<commit_message>
daily auto-refresh 2026-08-10 14:16
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -691,7 +691,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -10735,7 +10735,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-17 14:08
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -1600,7 +1600,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£500-£1K</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£200-£500</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2188,7 +2188,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£200-£500</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£200-£500</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£200-£500</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£200-£500</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£200-£500</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£200-£500</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£200-£500</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£100-£200</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£100-£200</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£100-£200</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>£100-£1K</t>
+          <t>£100-£200</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-17 14:39
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-18 16:42
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -859,7 +859,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Psyllium Husk Daily Fiber</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -4340,7 +4340,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Psyllium Husk Daily Fiber</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4681,7 +4681,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -5936,7 +5936,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -6020,12 +6020,12 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -8545,7 +8545,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -9044,7 +9044,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -9385,7 +9385,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
@@ -10371,7 +10371,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-19 17:35
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Spearmint</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4807,7 +4807,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Psyllium Husk Daily Fiber</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -6104,7 +6104,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Psyllium Husk Daily Fiber</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -6949,7 +6949,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -7075,7 +7075,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -7154,7 +7154,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -7322,7 +7322,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -7616,7 +7616,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -8545,7 +8545,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -8839,7 +8839,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
@@ -11505,7 +11505,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -12125,7 +12125,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -13153,7 +13153,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
@@ -14045,7 +14045,7 @@
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
@@ -14929,7 +14929,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
@@ -16355,7 +16355,7 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-20 07:00
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -6613,7 +6613,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -6949,7 +6949,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -7075,7 +7075,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -7453,7 +7453,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -8797,7 +8797,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -8839,7 +8839,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
@@ -9462,7 +9462,7 @@
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="inlineStr">
         <is>
-          <t>Psyllium Husk Daily Fiber</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
@@ -11505,7 +11505,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -12125,7 +12125,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -13595,7 +13595,7 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
@@ -14113,7 +14113,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
@@ -14895,7 +14895,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
@@ -15803,7 +15803,7 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-25 12:54
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -6403,7 +6403,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-31 08:49
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3799,7 +3799,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -6235,7 +6235,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -10589,7 +10589,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-31 08:51
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -607,7 +607,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -6235,7 +6235,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -8791,7 +8791,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-31 11:02
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -3085,7 +3085,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-04 08:53 (full-year creatives restored; +44 affiliate-centre slabs)
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1775" uniqueCount="769">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1777" uniqueCount="769">
   <si>
     <t>handle</t>
   </si>
@@ -5835,6 +5835,9 @@
       <c r="A128" t="s">
         <v>134</v>
       </c>
+      <c r="B128" t="s">
+        <v>268</v>
+      </c>
       <c r="D128" t="s">
         <v>277</v>
       </c>
@@ -6327,6 +6330,9 @@
     <row r="151" spans="1:8">
       <c r="A151" t="s">
         <v>157</v>
+      </c>
+      <c r="B151" t="s">
+        <v>268</v>
       </c>
       <c r="D151" t="s">
         <v>280</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-07 12:25
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Psyllium Husk Daily Fiber</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -7246,12 +7246,12 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Psyllium Husk Daily Fiber</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -7885,7 +7885,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">

</xml_diff>